<commit_message>
Fix venue identity, filters, and deadline display
</commit_message>
<xml_diff>
--- a/timeline_data.xlsx
+++ b/timeline_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="2025submit-2025conf" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="2025submit-2026conf" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="2026submit-2026conf" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="2026submit-2027conf" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025submit-2025conf" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025submit-2026conf" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026submit-2026conf" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026submit-2027conf" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -786,7 +786,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O48"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1698,7 +1698,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>csf</t>
+          <t>csfw</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1751,7 +1751,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>csf</t>
+          <t>csfw</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2923,12 +2923,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>recomb</t>
+          <t>cscw</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>RECOMB</t>
+          <t>CSCW</t>
         </is>
       </c>
       <c r="C35" t="n">
@@ -2939,37 +2939,32 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-05-14</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
-        </is>
-      </c>
-      <c r="J35" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
+          <t>2025-08-19</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Thessaloniki, Greece</t>
+          <t>Salt Lake City, UT, USA</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>http://recomb.org/recomb2026/</t>
+          <t>https://cscw.acm.org/2026/</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -2981,12 +2976,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>cscw</t>
+          <t>recomb</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CSCW</t>
+          <t>RECOMB</t>
         </is>
       </c>
       <c r="C36" t="n">
@@ -2997,32 +2992,37 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2025-05-14</t>
+          <t>2025-11-20</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>2025-08-19</t>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-05-26</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Salt Lake City, UT, USA</t>
+          <t>Thessaloniki, Greece</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>https://cscw.acm.org/2026/</t>
+          <t>http://recomb.org/recomb2026/</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -3034,12 +3034,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>recomb</t>
+          <t>icde</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>RECOMB</t>
+          <t>ICDE</t>
         </is>
       </c>
       <c r="C37" t="n">
@@ -3050,42 +3050,37 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2025-11-20</t>
+          <t>2025-06-18</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
-        </is>
-      </c>
-      <c r="J37" t="inlineStr">
-        <is>
-          <t>2026-02-25</t>
+          <t>2025-10-20</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>2026-05-26</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Thessaloniki, Greece</t>
+          <t>Montreal, Canada</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>http://recomb.org/recomb2026/</t>
+          <t>https://icde2026.github.io/</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>AoE</t>
+          <t>US Pacific</t>
         </is>
       </c>
     </row>
@@ -3104,16 +3099,16 @@
         <v>2026</v>
       </c>
       <c r="D38" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>2025-06-18</t>
+          <t>2025-10-27</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>2025-10-20</t>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -3145,53 +3140,53 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>icde</t>
+          <t>sigmetrics</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>ICDE</t>
+          <t>SIGMETRICS</t>
         </is>
       </c>
       <c r="C39" t="n">
         <v>2026</v>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>2025-10-27</t>
+          <t>2025-07-29</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>2026-02-23</t>
+          <t>2025-09-26</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>2026-05-04</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Montreal, Canada</t>
+          <t>Ann Arbor, MI, USA</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>https://icde2026.github.io/</t>
+          <t>https://www.sigmetrics.org/sigmetrics2026/</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>US Pacific</t>
+          <t>AoE</t>
         </is>
       </c>
     </row>
@@ -3210,16 +3205,16 @@
         <v>2026</v>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>2025-07-29</t>
+          <t>2025-10-14</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>2025-09-26</t>
+          <t>2025-12-12</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -3251,48 +3246,68 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>sigmetrics</t>
+          <t>aamas</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>SIGMETRICS</t>
+          <t>AAMAS</t>
         </is>
       </c>
       <c r="C41" t="n">
         <v>2026</v>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2025-10-14</t>
+          <t>2025-10-08</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>2025-10-01</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2025-11-21</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>2025-12-12</t>
+          <t>2025-12-22</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>2026-06-12</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Ann Arbor, MI, USA</t>
+          <t>Paphos, Cyprus</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>https://www.sigmetrics.org/sigmetrics2026/</t>
+          <t>https://cyprusconferences.org/aamas2026/</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3304,12 +3319,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>aamas</t>
+          <t>mobisys</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>AAMAS</t>
+          <t>MobiSys</t>
         </is>
       </c>
       <c r="C42" t="n">
@@ -3320,52 +3335,52 @@
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>2025-10-08</t>
+          <t>2025-12-05</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>2025-10-01</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>2025-11-21</t>
+          <t>2026-02-09</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>2025-11-25</t>
+          <t>2026-02-13</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>2025-12-22</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>2026-02-11</t>
+          <t>2026-04-13</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Paphos, Cyprus</t>
+          <t>Cambridge, UK</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>https://cyprusconferences.org/aamas2026/</t>
+          <t>https://www.sigmobile.org/mobisys/2026/</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3377,68 +3392,58 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>mobisys</t>
+          <t>cgo</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MobiSys</t>
+          <t>CGO</t>
         </is>
       </c>
       <c r="C43" t="n">
         <v>2026</v>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2025-12-05</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>2025-11-28</t>
+          <t>2025-09-11</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>2026-02-09</t>
+          <t>2025-10-21</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>2026-02-13</t>
+          <t>2025-10-23</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
-        </is>
-      </c>
-      <c r="J43" t="inlineStr">
-        <is>
-          <t>2026-04-13</t>
+          <t>2025-11-03</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-01-31</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-02-04</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Cambridge, UK</t>
+          <t>Sydney, Australia</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>https://www.sigmobile.org/mobisys/2026/</t>
+          <t>https://2026.cgo.org/</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -3450,58 +3455,43 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>cgo</t>
+          <t>icme</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CGO</t>
+          <t>ICME</t>
         </is>
       </c>
       <c r="C44" t="n">
         <v>2026</v>
       </c>
       <c r="D44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2025-09-11</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>2025-10-21</t>
-        </is>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>2025-10-23</t>
+          <t>2025-12-15</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2025-11-03</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-02-04</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Sydney, Australia</t>
-        </is>
-      </c>
-      <c r="N44" t="inlineStr">
-        <is>
-          <t>https://2026.cgo.org/</t>
+          <t>Bangkok, Thailand</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -3513,12 +3503,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>icme</t>
+          <t>fm</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>ICME</t>
+          <t>FM</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -3529,27 +3519,42 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2025-12-15</t>
+          <t>2025-12-02</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>2025-11-25</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Bangkok, Thailand</t>
+          <t>Tokyo, Japan</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>https://conf.researchr.org/home/fm-2026</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3561,12 +3566,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>fm</t>
+          <t>icpr</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>FM</t>
+          <t>ICPR</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -3577,42 +3582,27 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2025-12-02</t>
-        </is>
-      </c>
-      <c r="F46" t="inlineStr">
-        <is>
-          <t>2025-11-25</t>
+          <t>2025-12-21</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
-        </is>
-      </c>
-      <c r="J46" t="inlineStr">
-        <is>
-          <t>2026-02-23</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-08-17</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
-        </is>
-      </c>
-      <c r="N46" t="inlineStr">
-        <is>
-          <t>https://conf.researchr.org/home/fm-2026</t>
+          <t>Lyon, France</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -3624,12 +3614,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>icpr</t>
+          <t>caise</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>ICPR</t>
+          <t>CAiSE</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -3640,78 +3630,30 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2025-12-21</t>
+          <t>2025-11-28</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-06-12</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Lyon, France</t>
+          <t>Verona, Italy</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-    </row>
-    <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>caise</t>
-        </is>
-      </c>
-      <c r="B48" t="inlineStr">
-        <is>
-          <t>CAiSE</t>
-        </is>
-      </c>
-      <c r="C48" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D48" t="n">
-        <v>1</v>
-      </c>
-      <c r="E48" t="inlineStr">
-        <is>
-          <t>2025-11-28</t>
-        </is>
-      </c>
-      <c r="I48" t="inlineStr">
-        <is>
-          <t>2026-02-01</t>
-        </is>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>2026-06-08</t>
-        </is>
-      </c>
-      <c r="L48" t="inlineStr">
-        <is>
-          <t>2026-06-12</t>
-        </is>
-      </c>
-      <c r="M48" t="inlineStr">
-        <is>
-          <t>Verona, Italy</t>
-        </is>
-      </c>
-      <c r="O48" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -3728,7 +3670,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P54"/>
+  <dimension ref="A1:P53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4350,7 +4292,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>csf</t>
+          <t>csfw</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -4756,7 +4698,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>kdd</t>
+          <t>sigkdd</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -6097,7 +6039,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>hotchips</t>
+          <t>hot-chips</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -6329,12 +6271,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>fuzz-ieee</t>
+          <t>ieee-cec</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>FUZZ-IEEE</t>
+          <t>IEEE CEC</t>
         </is>
       </c>
       <c r="C43" t="n">
@@ -6387,12 +6329,12 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ieee-cec</t>
+          <t>soups</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>IEEE CEC</t>
+          <t>SOUPS</t>
         </is>
       </c>
       <c r="C44" t="n">
@@ -6403,37 +6345,37 @@
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>2026-01-31</t>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
-        </is>
-      </c>
-      <c r="J44" t="inlineStr">
-        <is>
-          <t>2026-04-15</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Maastricht, Netherlands</t>
+          <t>Hannover, Germany</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>https://attend.ieee.org/wcci-2026/</t>
+          <t>https://www.usenix.org/conference/soups2026/</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -6445,12 +6387,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>soups</t>
+          <t>icdar</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SOUPS</t>
+          <t>ICDAR</t>
         </is>
       </c>
       <c r="C45" t="n">
@@ -6461,40 +6403,25 @@
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>2026-02-19</t>
-        </is>
-      </c>
-      <c r="F45" t="inlineStr">
-        <is>
-          <t>2026-02-12</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>2026-05-19</t>
-        </is>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
+          <t>2026-02-27</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Hannover, Germany</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>https://www.usenix.org/conference/soups2026/</t>
-        </is>
-      </c>
-      <c r="O45" t="inlineStr">
+          <t>Vienna, Austria</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -6503,12 +6430,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>icdar</t>
+          <t>fg</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>ICDAR</t>
+          <t>FG</t>
         </is>
       </c>
       <c r="C46" t="n">
@@ -6519,22 +6446,22 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>2026-02-27</t>
+          <t>2026-01-09</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-05-25</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-05-29</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Vienna, Austria</t>
+          <t>Kyoto, Japan</t>
         </is>
       </c>
       <c r="P46" t="inlineStr">
@@ -6546,12 +6473,12 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>fg</t>
+          <t>bmvc</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>FG</t>
+          <t>BMVC</t>
         </is>
       </c>
       <c r="C47" t="n">
@@ -6562,22 +6489,22 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>2026-01-09</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>2026-05-25</t>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>2026-05-29</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Kyoto, Japan</t>
+          <t>TBD</t>
         </is>
       </c>
       <c r="P47" t="inlineStr">
@@ -6589,12 +6516,12 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>bmvc</t>
+          <t>iceccs</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>BMVC</t>
+          <t>ICECCS</t>
         </is>
       </c>
       <c r="C48" t="n">
@@ -6605,25 +6532,45 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>2026-11-23</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-24</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>2026-11-26</t>
+          <t>Brisbane, Australia</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="P48" t="inlineStr">
+          <t>https://easychair.org/conferences?conf=iceccs2026</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>
@@ -6632,12 +6579,12 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>iceccs</t>
+          <t>mobihoc</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>ICECCS</t>
+          <t>MobiHoc</t>
         </is>
       </c>
       <c r="C49" t="n">
@@ -6648,22 +6595,27 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
-        </is>
-      </c>
-      <c r="F49" t="inlineStr">
-        <is>
-          <t>2026-06-29</t>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2026-07-26</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-30</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -6673,17 +6625,17 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>2026-11-24</t>
+          <t>2026-11-26</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Brisbane, Australia</t>
+          <t>Tokyo, Japan</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>https://easychair.org/conferences?conf=iceccs2026</t>
+          <t>https://sigmobile.org/mobihoc/2026/</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -6695,12 +6647,12 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>mobihoc</t>
+          <t>cikm</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>MobiHoc</t>
+          <t>CIKM</t>
         </is>
       </c>
       <c r="C50" t="n">
@@ -6711,47 +6663,32 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>2026-07-26</t>
-        </is>
-      </c>
-      <c r="H50" t="inlineStr">
-        <is>
-          <t>2026-08-23</t>
+          <t>2026-05-23</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>2026-09-30</t>
-        </is>
-      </c>
-      <c r="J50" t="inlineStr">
-        <is>
-          <t>2026-09-30</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>2026-11-23</t>
+          <t>2026-11-07</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>2026-11-26</t>
+          <t>2026-11-11</t>
         </is>
       </c>
       <c r="M50" t="inlineStr">
         <is>
-          <t>Tokyo, Japan</t>
-        </is>
-      </c>
-      <c r="N50" t="inlineStr">
-        <is>
-          <t>https://sigmobile.org/mobihoc/2026/</t>
+          <t>Rome, Italy</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
@@ -6763,12 +6700,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>cikm</t>
+          <t>icdm</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CIKM</t>
+          <t>ICDM</t>
         </is>
       </c>
       <c r="C51" t="n">
@@ -6779,32 +6716,32 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>2026-05-23</t>
-        </is>
-      </c>
-      <c r="F51" t="inlineStr">
-        <is>
-          <t>2026-05-16</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>2026-11-07</t>
+          <t>2026-11-12</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>2026-11-11</t>
+          <t>2026-11-15</t>
         </is>
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>Rome, Italy</t>
+          <t>Shenyang, China</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
@@ -6816,12 +6753,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>icdm</t>
+          <t>icws</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ICDM</t>
+          <t>ICWS</t>
         </is>
       </c>
       <c r="C52" t="n">
@@ -6832,32 +6769,27 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-03-22</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="J52" t="inlineStr">
-        <is>
-          <t>2026-09-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>2026-11-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>2026-11-15</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="M52" t="inlineStr">
         <is>
-          <t>Shenyang, China</t>
+          <t>Sydney, Australia</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
@@ -6869,12 +6801,12 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>icws</t>
+          <t>icsoc</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>ICWS</t>
+          <t>ICSOC</t>
         </is>
       </c>
       <c r="C53" t="n">
@@ -6885,78 +6817,30 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>2026-03-22</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-12-01</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-12-04</t>
         </is>
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>Sydney, Australia</t>
+          <t>Lodz, Poland</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
-        <is>
-          <t>AoE</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>icsoc</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>ICSOC</t>
-        </is>
-      </c>
-      <c r="C54" t="n">
-        <v>2026</v>
-      </c>
-      <c r="D54" t="n">
-        <v>1</v>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>2026-07-19</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>2026-09-13</t>
-        </is>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>2026-12-01</t>
-        </is>
-      </c>
-      <c r="L54" t="inlineStr">
-        <is>
-          <t>2026-12-04</t>
-        </is>
-      </c>
-      <c r="M54" t="inlineStr">
-        <is>
-          <t>Lodz, Poland</t>
-        </is>
-      </c>
-      <c r="O54" t="inlineStr">
         <is>
           <t>AoE</t>
         </is>

</xml_diff>